<commit_message>
Mistakes to get solution of it
</commit_message>
<xml_diff>
--- a/School_Data.xlsx
+++ b/School_Data.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2535,20 +2535,16 @@
       <c r="A47" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>1679428506</t>
-        </is>
+      <c r="B47" t="n">
+        <v>1679428506</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
           <t>الاشكال والانماط</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="D47" t="n">
+        <v>2</v>
       </c>
       <c r="E47" t="n">
         <v>2</v>
@@ -2611,6 +2607,45 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1679428506</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>النقود</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>مرحبًا بك! إذا كنت بحاجة إلى أي مساعدة أو استفسار حول المحتوى التعليمي أو أي موضوع آخر، فلا تتردد في طرحه. أنا هنا لمساعدتك.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>غير معروف</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-04-07 09:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: enhance Arabic PDF generation and fix layout issues in report pdfs
</commit_message>
<xml_diff>
--- a/School_Data.xlsx
+++ b/School_Data.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2956,20 +2956,16 @@
       <c r="A53" t="n">
         <v>52</v>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>1679428506</t>
-        </is>
+      <c r="B53" t="n">
+        <v>1679428506</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
           <t>الوقت</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="D53" t="n">
+        <v>1</v>
       </c>
       <c r="E53" t="n">
         <v>2</v>
@@ -3035,6 +3031,100 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1679428506</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>الطرح البسيط</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>### خطة درس أولية: 'الطرح البسيط'
+#### الموضوع: فهم مفهوم الطرح كأخذ جزء من الكل
+#### الفئة المستهدفة: الطلاب في الصف الأول الابتدائي
+#### المدة: 40 دقيقة
+#### الفجوة التعليمية: 25.0%
+#### اتجاه الأداء: مستقر (بداية)
+---
+#### **الأهداف التعليمية:**
+1. فهم مفهوم الطرح كأخذ جزء من الكل.
+2. تعزيز مهارات الطرح من خلال الأنشطة التفاعلية.
+3. تطوير التفكير النقدي لدى الطلاب من خلال الممارسة العملية.
+---
+### **نشاط اللعبة التعليمية: "محطات الطرح"**
+#### **المرحلة 1: مقدمة (5 دقائق)**
+- يبدأ المعلم بشرح بسيط لمفهوم الطرح من خلال استخدام أمثلة مرئية (مثل تفاحة معروضة، وطرح عدد منها).
+- يوضح الفكرة بأن الطرح يعني أخذ جزء من الكل.
+#### **المرحلة 2: تقسيم الطلاب إلى مجموعات (5 دقائق)**
+- يقسم المعلم الطلاب إلى مجموعات صغيرة (4 طلاب في كل مجموعة).
+- يقدم لكل مجموعة بطاقة تحتوي على مسألة طرح بسيطة (مثل 5 - 2).
+#### **المرحلة 3: محطات التعلم (25 دقيقة)**
+- يتم إعداد 4 محطات تعليمية مختلفة، حيث يقضي الطلاب 5 دقائق في كل محطة:
+##### **المحطة 1: محطة الفواكه**
+- استخدام كرات ملونة أو فواكه مصنوعة من الورق.
+- يقوم الطلاب بأخذ عدد معين من الكرات، ثم يطرحون منها عددًا محددًا.
+- يشرح كل طالب لزملائه ما حدث.
+##### **المحطة 2: محطة الأرقام**
+- استخدام بطاقات الأرقام.
+- يقوم الطلاب بسحب بطاقتين (مثل 7 و3)، ثم يقومون بطرح الرقمين باستخدام البطاقات.
+- يشجع المعلم الطلاب على مناقشة النتائج مع بعضهم.
+##### **المحطة 3: محطة القصص**
+- يقدم المعلم قصة قصيرة تتضمن عملية طرح.
+- يطلب من الطلاب تمثيل القصة من خلال اللعب، حيث يقوم أحدهم بأخذ جزء من الكل (مثل: "كان هناك 6 طيور في الشجرة، طار 2 منهم، كم تبقى؟").
+##### **المحطة 4: محطة اللوحات**
+- يقدم المعلم لوحات بيضاء وأقلام.
+- يقوم الطلاب بإنشاء معادلات طرح خاصة بهم ورسم صور توضح الفكرة.
+- يسمح للطلاب بمشاركة لوحاتهم مع باقي المجموعات.
+#### **المرحلة 4: تقييم التعلم (5 دقائق)**
+- يقوم المعلم بجمع المجموعات معًا ويسألهم أسئلة تفاعلية حول ما تعلموه.
+- يمكن استخدام أسئلة مثل:
+  - ما هو الطرح؟
+  - كيف يمكننا استخدام الطرح في حياتنا اليومية؟
+---
+### **المواد المطلوبة:**
+- كرات ملونة أو فواكه ورقية.
+- بطاقات أرقام.
+- بطاقات مع مسائل طرح.
+- لوحات بيضاء وأقلام.
+### **ملاحظات:**
+- التأكد من توفير بيئة تعليمية إيجابية وداعمة.
+- يجب أن تكون الأنشطة ممتعة وتشجع على التعاون بين الطلاب.
+- يمكن للمعلم تعديل المحطات حسب احتياجات الطلاب ومستوى فهمهم.
+### **التقييم والمتابعة:**
+- استخدام ملاحظات المعلم خلال النشاط لتحديد مدى فهم الطلاب للمفهوم.
+- يمكن إجراء اختبار قصير في الدروس التالية لتقييم التقدم المحرز في فهم الطرح.
+---
+هذه الخطة مصممة لتعزيز فهم الطلاب لمفهوم الطرح من خلال الأنشطة العملية والتفاعلية، مما يساعد في تقليل الفجوة التعليمية وتعزيز المشاركة.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>غير معروف</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-04-12 15:29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>